<commit_message>
Actualizar datos 2026 (2026-04-10)
</commit_message>
<xml_diff>
--- a/data/asistencia/Charros 2026.xlsx
+++ b/data/asistencia/Charros 2026.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="53">
   <si>
     <t>Reporte de disponibilidad por zona</t>
   </si>
@@ -97,79 +97,79 @@
     <t>Gourmet</t>
   </si>
   <si>
-    <t>14.87%</t>
+    <t>24.57%</t>
   </si>
   <si>
     <t>Lateral Preferente Primera Base</t>
   </si>
   <si>
-    <t>97.16%</t>
+    <t>97.67%</t>
   </si>
   <si>
     <t>Lateral Preferente Tercera Base</t>
   </si>
   <si>
-    <t>96.64%</t>
+    <t>97.42%</t>
   </si>
   <si>
     <t>Lateral Primera Base</t>
   </si>
   <si>
-    <t>80.61%</t>
+    <t>84.96%</t>
   </si>
   <si>
     <t>Lateral Tercera Base</t>
   </si>
   <si>
-    <t>48.43%</t>
+    <t>56.62%</t>
   </si>
   <si>
     <t>Planta Alta Central</t>
   </si>
   <si>
-    <t>57.62%</t>
+    <t>60.87%</t>
   </si>
   <si>
     <t>Planta Alta Lateral Primera Base</t>
   </si>
   <si>
-    <t>33.36%</t>
+    <t>39.91%</t>
   </si>
   <si>
     <t>Planta Alta Lateral Tercera Base</t>
   </si>
   <si>
-    <t>22.15%</t>
+    <t>28.58%</t>
   </si>
   <si>
     <t>Planta Baja</t>
   </si>
   <si>
-    <t>97.20%</t>
+    <t>97.49%</t>
   </si>
   <si>
     <t>Premier 1ra-3ra</t>
   </si>
   <si>
-    <t>93.97%</t>
+    <t>96.99%</t>
   </si>
   <si>
     <t>Premier Home</t>
   </si>
   <si>
-    <t>99.43%</t>
+    <t>99.62%</t>
   </si>
   <si>
     <t>SUITES</t>
   </si>
   <si>
-    <t>4.42%</t>
+    <t>7.53%</t>
   </si>
   <si>
     <t>TOTALES</t>
   </si>
   <si>
-    <t>60.84%</t>
+    <t>64.96%</t>
   </si>
 </sst>
 </file>
@@ -812,7 +812,7 @@
         <v>23</v>
       </c>
       <c r="C8" s="7">
-        <v>50</v>
+        <v>112</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>23</v>
@@ -854,10 +854,10 @@
         <v>639</v>
       </c>
       <c r="Q8" s="7">
-        <v>95</v>
+        <v>157</v>
       </c>
       <c r="R8" s="7">
-        <v>544</v>
+        <v>482</v>
       </c>
       <c r="S8" s="8" t="s">
         <v>28</v>
@@ -871,7 +871,7 @@
         <v>23</v>
       </c>
       <c r="C9" s="7">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D9" s="7">
         <v>23</v>
@@ -913,10 +913,10 @@
         <v>387</v>
       </c>
       <c r="Q9" s="7">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="R9" s="7">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="S9" s="8" t="s">
         <v>30</v>
@@ -930,7 +930,7 @@
         <v>23</v>
       </c>
       <c r="C10" s="7">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D10" s="7">
         <v>21</v>
@@ -972,10 +972,10 @@
         <v>387</v>
       </c>
       <c r="Q10" s="7">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="R10" s="7">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="S10" s="8" t="s">
         <v>32</v>
@@ -989,7 +989,7 @@
         <v>23</v>
       </c>
       <c r="C11" s="7">
-        <v>559</v>
+        <v>616</v>
       </c>
       <c r="D11" s="7">
         <v>84</v>
@@ -1031,10 +1031,10 @@
         <v>1310</v>
       </c>
       <c r="Q11" s="7">
-        <v>1056</v>
+        <v>1113</v>
       </c>
       <c r="R11" s="7">
-        <v>254</v>
+        <v>197</v>
       </c>
       <c r="S11" s="8" t="s">
         <v>34</v>
@@ -1048,7 +1048,7 @@
         <v>23</v>
       </c>
       <c r="C12" s="7">
-        <v>301</v>
+        <v>413</v>
       </c>
       <c r="D12" s="7">
         <v>43</v>
@@ -1084,16 +1084,16 @@
         <v>23</v>
       </c>
       <c r="O12" s="7">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="P12" s="7">
         <v>1307</v>
       </c>
       <c r="Q12" s="7">
-        <v>633</v>
+        <v>740</v>
       </c>
       <c r="R12" s="7">
-        <v>674</v>
+        <v>567</v>
       </c>
       <c r="S12" s="8" t="s">
         <v>36</v>
@@ -1107,7 +1107,7 @@
         <v>23</v>
       </c>
       <c r="C13" s="7">
-        <v>554</v>
+        <v>601</v>
       </c>
       <c r="D13" s="7">
         <v>86</v>
@@ -1149,10 +1149,10 @@
         <v>1444</v>
       </c>
       <c r="Q13" s="7">
-        <v>832</v>
+        <v>879</v>
       </c>
       <c r="R13" s="7">
-        <v>612</v>
+        <v>565</v>
       </c>
       <c r="S13" s="8" t="s">
         <v>38</v>
@@ -1162,11 +1162,11 @@
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>23</v>
+      <c r="B14" s="7">
+        <v>4</v>
       </c>
       <c r="C14" s="7">
-        <v>299</v>
+        <v>365</v>
       </c>
       <c r="D14" s="7">
         <v>57</v>
@@ -1208,10 +1208,10 @@
         <v>1070</v>
       </c>
       <c r="Q14" s="7">
-        <v>357</v>
+        <v>427</v>
       </c>
       <c r="R14" s="7">
-        <v>713</v>
+        <v>643</v>
       </c>
       <c r="S14" s="8" t="s">
         <v>40</v>
@@ -1225,7 +1225,7 @@
         <v>23</v>
       </c>
       <c r="C15" s="7">
-        <v>212</v>
+        <v>282</v>
       </c>
       <c r="D15" s="7">
         <v>25</v>
@@ -1267,10 +1267,10 @@
         <v>1088</v>
       </c>
       <c r="Q15" s="7">
-        <v>241</v>
+        <v>311</v>
       </c>
       <c r="R15" s="7">
-        <v>847</v>
+        <v>777</v>
       </c>
       <c r="S15" s="8" t="s">
         <v>42</v>
@@ -1284,13 +1284,13 @@
         <v>23</v>
       </c>
       <c r="C16" s="7">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="D16" s="7">
         <v>119</v>
       </c>
       <c r="E16" s="7">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>23</v>
@@ -1320,16 +1320,16 @@
         <v>23</v>
       </c>
       <c r="O16" s="7">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="P16" s="7">
         <v>1036</v>
       </c>
       <c r="Q16" s="7">
-        <v>1007</v>
+        <v>1010</v>
       </c>
       <c r="R16" s="7">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="S16" s="8" t="s">
         <v>44</v>
@@ -1343,7 +1343,7 @@
         <v>23</v>
       </c>
       <c r="C17" s="7">
-        <v>531</v>
+        <v>558</v>
       </c>
       <c r="D17" s="7">
         <v>107</v>
@@ -1385,10 +1385,10 @@
         <v>896</v>
       </c>
       <c r="Q17" s="7">
-        <v>842</v>
+        <v>869</v>
       </c>
       <c r="R17" s="7">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="S17" s="8" t="s">
         <v>46</v>
@@ -1402,7 +1402,7 @@
         <v>23</v>
       </c>
       <c r="C18" s="7">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D18" s="7">
         <v>45</v>
@@ -1444,10 +1444,10 @@
         <v>530</v>
       </c>
       <c r="Q18" s="7">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="R18" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S18" s="8" t="s">
         <v>48</v>
@@ -1482,7 +1482,7 @@
         <v>23</v>
       </c>
       <c r="J19" s="7">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>23</v>
@@ -1503,10 +1503,10 @@
         <v>770</v>
       </c>
       <c r="Q19" s="7">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="R19" s="7">
-        <v>736</v>
+        <v>712</v>
       </c>
       <c r="S19" s="8" t="s">
         <v>50</v>

</xml_diff>